<commit_message>
docs: update Excel template with multi-site support
Template now has 3 sheets:
- tek_alan: single-site format (10 species, 8 columns)
- coklu_alan: multi-site format (3 sites, 15 rows, Site column)
- KULLANIM: usage guide with R code examples for batch_analysis()
</commit_message>
<xml_diff>
--- a/inst/templates/taxdiv_template.xlsx
+++ b/inst/templates/taxdiv_template.xlsx
@@ -6,13 +6,15 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="taxdiv_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tek_alan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="coklu_alan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="KULLANIM" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t xml:space="preserve">Species</t>
   </si>
@@ -104,12 +106,6 @@
     <t xml:space="preserve">Cedrus</t>
   </si>
   <si>
-    <t xml:space="preserve">Pinus brutia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quercus infectoria</t>
-  </si>
-  <si>
     <t xml:space="preserve">Carpinus betulus</t>
   </si>
   <si>
@@ -119,7 +115,7 @@
     <t xml:space="preserve">Betulaceae</t>
   </si>
   <si>
-    <t xml:space="preserve">Acer campestre</t>
+    <t xml:space="preserve">Acer platanoides</t>
   </si>
   <si>
     <t xml:space="preserve">Acer</t>
@@ -129,6 +125,102 @@
   </si>
   <si>
     <t xml:space="preserve">Sapindales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tilia tomentosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tilia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malvaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malvales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorbus torminalis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorbus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rosaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rosales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alan_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alan_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alan_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEK ALAN ANALIZI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tek bir ornek alandaki turlerin cesitlilik analizi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gerekli sutunlar:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species, Genus, Family, Order (+ Class, Phylum, Kingdom istege bagli)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abundance sutunu:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Her tur icin birey sayisi (sayisal deger olmali)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">COKLU ALAN ANALIZI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Birden fazla ornek alanin ayri ayri analizi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ek sutun:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site (veya Alan veya Plot) sutunu ekleyin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site sutun isimleri:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site, site, Alan, alan, Plot, plot (otomatik algilanir)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R KODU - Tek Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">library(taxdiv)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">library(readxl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">veri &lt;- as.data.frame(read_excel("dosya.xlsx", sheet = "tek_alan"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sonuc &lt;- batch_analysis(veri)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R KODU - Coklu Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">veri &lt;- as.data.frame(read_excel("dosya.xlsx", sheet = "coklu_alan"))</t>
   </si>
 </sst>
 </file>
@@ -136,7 +228,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -155,8 +247,19 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -175,7 +278,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE3F2FD"/>
+        <fgColor rgb="FF1B5E20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -189,44 +297,58 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF1B5E20"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF1B5E20"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF1B5E20"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF1B5E20"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFC8E6C9"/>
       </left>
       <right style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFC8E6C9"/>
       </right>
       <top style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFC8E6C9"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FFC8E6C9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -518,13 +640,13 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="25.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="12.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -715,39 +837,39 @@
         <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>19</v>
@@ -759,21 +881,21 @@
         <v>14</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>19</v>
@@ -785,21 +907,21 @@
         <v>14</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>19</v>
@@ -811,7 +933,636 @@
         <v>14</v>
       </c>
       <c r="H11" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="16.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="30.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="70.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add numeric codes example sheet to Excel template
New 'sayisal_kodlar' sheet shows that taxonomic ranks can be
entered as numbers instead of text names. Same grouping logic
applies — species sharing a rank get the same number.
KULLANIM sheet updated with numeric code instructions.
</commit_message>
<xml_diff>
--- a/inst/templates/taxdiv_template.xlsx
+++ b/inst/templates/taxdiv_template.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="tek_alan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="coklu_alan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="KULLANIM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="sayisal_kodlar" sheetId="4" state="visible" r:id="rId3"/>
+    <sheet name="KULLANIM" sheetId="5" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t xml:space="preserve">Species</t>
   </si>
@@ -221,6 +222,24 @@
   </si>
   <si>
     <t xml:space="preserve">veri &lt;- as.data.frame(read_excel("dosya.xlsx", sheet = "coklu_alan"))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAYISAL KOD KULLANIMI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taksonomik kategoriler icin isim yerine sayi kullanabilirsiniz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kural:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayni gruba ait turler AYNI NUMARAYI almalidirlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ornek:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pinus ve Cedrus ayni Familya ise ikisi de Family=1 olmali</t>
   </si>
 </sst>
 </file>
@@ -228,7 +247,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -254,12 +273,18 @@
       <b/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Courier New"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -274,6 +299,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -327,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -341,13 +381,25 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1433,31 +1485,517 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="24.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="12.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="30.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="70.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="8" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1470,26 +2008,26 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="8" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="9" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="9" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1502,66 +2040,98 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B13" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="s">
+    <row r="14">
+      <c r="A14" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B14" s="11" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="s">
+    <row r="15">
+      <c r="A15" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B15" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="s">
+    <row r="16">
+      <c r="A16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B16" s="11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="s">
+    <row r="17">
+      <c r="A17" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B17" s="11" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="s">
+    <row r="18">
+      <c r="A18" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B18" s="11" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="s">
+    <row r="19">
+      <c r="A19" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B19" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="s">
+    <row r="20">
+      <c r="A20" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B20" s="11" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>